<commit_message>
updated partslist for first delivery of material
</commit_message>
<xml_diff>
--- a/cad/rig_v2/Partlist_v2.xlsx
+++ b/cad/rig_v2/Partlist_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tallA\Repos\VolumanXR\hardware-capture\cad\rig_v2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aldi\Repos\VolumanXR\hardware-capture\cad\rig_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86E5511-8C2D-4988-B07A-BCE014C50EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EB62D37-85DB-4F05-B37F-755D6063AD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-10785" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stückliste" sheetId="1" r:id="rId1"/>
@@ -1180,14 +1180,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I128"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="30.85546875" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1400,7 +1400,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -1469,7 +1469,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -1492,7 +1492,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -1515,7 +1515,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -1584,7 +1584,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
@@ -1600,6 +1600,9 @@
       <c r="F18" s="1">
         <v>4</v>
       </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
       <c r="H18" s="1" t="s">
         <v>87</v>
       </c>
@@ -1607,7 +1610,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
@@ -1623,6 +1626,9 @@
       <c r="F19" s="1">
         <v>29</v>
       </c>
+      <c r="G19">
+        <v>29</v>
+      </c>
       <c r="H19" s="1" t="s">
         <v>87</v>
       </c>
@@ -1630,7 +1636,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1647,7 +1653,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
@@ -1663,6 +1669,9 @@
       <c r="F21" s="1">
         <v>22</v>
       </c>
+      <c r="G21">
+        <v>22</v>
+      </c>
       <c r="H21" s="1" t="s">
         <v>87</v>
       </c>
@@ -1670,7 +1679,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>29</v>
       </c>
@@ -1693,7 +1702,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>30</v>
       </c>
@@ -1719,7 +1728,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>31</v>
       </c>
@@ -1736,7 +1745,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>32</v>
       </c>
@@ -1756,7 +1765,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>33</v>
       </c>
@@ -1772,6 +1781,9 @@
       <c r="F26" s="1">
         <v>2</v>
       </c>
+      <c r="G26">
+        <v>2</v>
+      </c>
       <c r="H26" s="1" t="s">
         <v>87</v>
       </c>
@@ -1779,7 +1791,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>34</v>
       </c>
@@ -1795,6 +1807,9 @@
       <c r="F27" s="1">
         <v>1</v>
       </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
       <c r="H27" s="1" t="s">
         <v>87</v>
       </c>
@@ -1802,7 +1817,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>35</v>
       </c>
@@ -1822,7 +1837,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>36</v>
       </c>
@@ -1842,13 +1857,13 @@
         <v>91</v>
       </c>
     </row>
-    <row r="122" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="68.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="123" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="124" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="125" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="126" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="127" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="128" ht="68.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>